<commit_message>
Document completed Employee and EmployeeType live acceptance
</commit_message>
<xml_diff>
--- a/docs/bulk-upload/05-employees.xlsx
+++ b/docs/bulk-upload/05-employees.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R6233ddb47b914a2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="R22369233c6eb49b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Employees" sheetId="1" r:id="R066819db65994aa8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="2" r:id="R240db6b4398943e0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1017,7 +1017,7 @@
         <x:v>Availability</x:v>
       </x:c>
       <x:c r="B2" s="12" t="str">
-        <x:v>Employee import is implemented locally with automated tests. Render deployment and authenticated HTTP acceptance remain pending.</x:v>
+        <x:v>Employee import is deployed. CSV import, skip replay, code recoding and database checks passed on 11 September 2026. See the UI guide for test coverage.</x:v>
       </x:c>
       <x:c r="C2" s="11"/>
       <x:c r="D2" s="11"/>

</xml_diff>